<commit_message>
update(): novo train com maximização de parametros
</commit_message>
<xml_diff>
--- a/src - analytics/top_50_previsoes.xlsx
+++ b/src - analytics/top_50_previsoes.xlsx
@@ -707,7 +707,7 @@
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
       <c r="AH2" t="n">
-        <v>0.650338236848668</v>
+        <v>0.6513504976142183</v>
       </c>
     </row>
     <row r="3">
@@ -817,7 +817,7 @@
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>
       <c r="AH3" t="n">
-        <v>0.6467077820108499</v>
+        <v>0.6471949453105131</v>
       </c>
     </row>
     <row r="4">
@@ -1029,7 +1029,7 @@
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
       <c r="AH5" t="n">
-        <v>0.631316291579607</v>
+        <v>0.631341778141238</v>
       </c>
     </row>
     <row r="6">
@@ -1245,7 +1245,7 @@
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
       <c r="AH7" t="n">
-        <v>0.6277049815372435</v>
+        <v>0.6276606671559726</v>
       </c>
     </row>
     <row r="8">
@@ -1355,7 +1355,7 @@
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
       <c r="AH8" t="n">
-        <v>0.6171617140402206</v>
+        <v>0.6166872006018518</v>
       </c>
     </row>
     <row r="9">
@@ -1571,7 +1571,7 @@
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="inlineStr"/>
       <c r="AH10" t="n">
-        <v>0.6094643480276508</v>
+        <v>0.6099515113273141</v>
       </c>
     </row>
     <row r="11">
@@ -1681,7 +1681,7 @@
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="inlineStr"/>
       <c r="AH11" t="n">
-        <v>0.6038305573573519</v>
+        <v>0.6033175731087355</v>
       </c>
     </row>
     <row r="12">
@@ -1791,7 +1791,7 @@
       <c r="AF12" t="inlineStr"/>
       <c r="AG12" t="inlineStr"/>
       <c r="AH12" t="n">
-        <v>0.5935210119967944</v>
+        <v>0.5934766976155235</v>
       </c>
     </row>
     <row r="13">
@@ -2113,7 +2113,7 @@
       <c r="AF15" t="inlineStr"/>
       <c r="AG15" t="inlineStr"/>
       <c r="AH15" t="n">
-        <v>0.5850650024355742</v>
+        <v>0.5849721452927171</v>
       </c>
     </row>
     <row r="16">
@@ -2223,7 +2223,7 @@
       <c r="AF16" t="inlineStr"/>
       <c r="AG16" t="inlineStr"/>
       <c r="AH16" t="n">
-        <v>0.5843281535153161</v>
+        <v>0.5846364541647084</v>
       </c>
     </row>
     <row r="17">
@@ -2439,7 +2439,7 @@
       <c r="AF18" t="inlineStr"/>
       <c r="AG18" t="inlineStr"/>
       <c r="AH18" t="n">
-        <v>0.5767584356561199</v>
+        <v>0.5767641174743018</v>
       </c>
     </row>
     <row r="19">
@@ -2659,7 +2659,7 @@
       <c r="AF20" t="inlineStr"/>
       <c r="AG20" t="inlineStr"/>
       <c r="AH20" t="n">
-        <v>0.5740312665957932</v>
+        <v>0.5739869522145223</v>
       </c>
     </row>
     <row r="21">
@@ -2775,17 +2775,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>prospol01</t>
+          <t>willima07</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>OLIVIER-MAXENCE PROSPER</t>
+          <t>MARK WILLIAMS</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PF</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -2793,105 +2793,107 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>DAL</t>
+          <t>CHO</t>
         </is>
       </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H22" t="n">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="I22" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="J22" t="n">
-        <v>336</v>
+        <v>508</v>
       </c>
       <c r="K22" t="n">
-        <v>121</v>
+        <v>242</v>
       </c>
       <c r="L22" t="n">
         <v>22</v>
       </c>
       <c r="M22" t="n">
-        <v>79</v>
+        <v>184</v>
       </c>
       <c r="N22" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="O22" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="P22" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="Q22" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="R22" t="n">
-        <v>0.6830000000000001</v>
+        <v>0.719</v>
       </c>
       <c r="S22" t="n">
-        <v>0.458</v>
-      </c>
-      <c r="T22" t="n">
-        <v>0.289</v>
-      </c>
+        <v>0.649</v>
+      </c>
+      <c r="T22" t="inlineStr"/>
       <c r="U22" t="n">
-        <v>0.385</v>
+        <v>0.649</v>
       </c>
       <c r="V22" t="n">
-        <v>267</v>
+        <v>607</v>
       </c>
       <c r="W22" t="n">
-        <v>6.675</v>
+        <v>31.94736842105263</v>
       </c>
       <c r="X22" t="n">
-        <v>0.7946428571428571</v>
+        <v>1.19488188976378</v>
       </c>
       <c r="Y22" t="n">
-        <v>267</v>
+        <v>31.94736842105263</v>
       </c>
       <c r="Z22" t="n">
-        <v>0.01535806729939603</v>
+        <v>0.05250865051903114</v>
       </c>
       <c r="AA22" t="n">
-        <v>28.60714285714285</v>
+        <v>43.01574803149607</v>
       </c>
       <c r="AB22" t="n">
-        <v>5.5</v>
+        <v>11</v>
       </c>
       <c r="AC22" t="inlineStr">
         <is>
-          <t>Nivel 2: Average</t>
-        </is>
-      </c>
-      <c r="AD22" t="inlineStr"/>
-      <c r="AE22" t="inlineStr"/>
+          <t>Nivel 4: Elite</t>
+        </is>
+      </c>
+      <c r="AD22" t="n">
+        <v>978</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>-371</v>
+      </c>
       <c r="AF22" t="inlineStr"/>
       <c r="AG22" t="inlineStr"/>
       <c r="AH22" t="n">
-        <v>0.5721092020284226</v>
+        <v>0.5717725538363014</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>willima07</t>
+          <t>prospol01</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MARK WILLIAMS</t>
+          <t>OLIVIER-MAXENCE PROSPER</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>PF</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -2899,91 +2901,89 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>CHO</t>
+          <t>DAL</t>
         </is>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H23" t="n">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="I23" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="J23" t="n">
-        <v>508</v>
+        <v>336</v>
       </c>
       <c r="K23" t="n">
-        <v>242</v>
+        <v>121</v>
       </c>
       <c r="L23" t="n">
         <v>22</v>
       </c>
       <c r="M23" t="n">
-        <v>184</v>
+        <v>79</v>
       </c>
       <c r="N23" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="O23" t="n">
+        <v>4</v>
+      </c>
+      <c r="P23" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q23" t="n">
         <v>20</v>
       </c>
-      <c r="P23" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>50</v>
-      </c>
       <c r="R23" t="n">
-        <v>0.719</v>
+        <v>0.6830000000000001</v>
       </c>
       <c r="S23" t="n">
-        <v>0.649</v>
-      </c>
-      <c r="T23" t="inlineStr"/>
+        <v>0.458</v>
+      </c>
+      <c r="T23" t="n">
+        <v>0.289</v>
+      </c>
       <c r="U23" t="n">
-        <v>0.649</v>
+        <v>0.385</v>
       </c>
       <c r="V23" t="n">
-        <v>607</v>
+        <v>267</v>
       </c>
       <c r="W23" t="n">
-        <v>31.94736842105263</v>
+        <v>6.675</v>
       </c>
       <c r="X23" t="n">
-        <v>1.19488188976378</v>
+        <v>0.7946428571428571</v>
       </c>
       <c r="Y23" t="n">
-        <v>31.94736842105263</v>
+        <v>267</v>
       </c>
       <c r="Z23" t="n">
-        <v>0.05250865051903114</v>
+        <v>0.01535806729939603</v>
       </c>
       <c r="AA23" t="n">
-        <v>43.01574803149607</v>
+        <v>28.60714285714285</v>
       </c>
       <c r="AB23" t="n">
-        <v>11</v>
+        <v>5.5</v>
       </c>
       <c r="AC23" t="inlineStr">
         <is>
-          <t>Nivel 4: Elite</t>
-        </is>
-      </c>
-      <c r="AD23" t="n">
-        <v>978</v>
-      </c>
-      <c r="AE23" t="n">
-        <v>-371</v>
-      </c>
+          <t>Nivel 2: Average</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr"/>
       <c r="AF23" t="inlineStr"/>
       <c r="AG23" t="inlineStr"/>
       <c r="AH23" t="n">
-        <v>0.5717725538363014</v>
+        <v>0.5714323727601299</v>
       </c>
     </row>
     <row r="24">
@@ -3091,7 +3091,7 @@
       <c r="AF24" t="inlineStr"/>
       <c r="AG24" t="inlineStr"/>
       <c r="AH24" t="n">
-        <v>0.5695564455146348</v>
+        <v>0.5693445788264314</v>
       </c>
     </row>
     <row r="25">
@@ -3307,7 +3307,7 @@
       <c r="AF26" t="inlineStr"/>
       <c r="AG26" t="inlineStr"/>
       <c r="AH26" t="n">
-        <v>0.5665517955243703</v>
+        <v>0.5664620258766737</v>
       </c>
     </row>
     <row r="27">
@@ -3417,7 +3417,7 @@
       <c r="AF27" t="inlineStr"/>
       <c r="AG27" t="inlineStr"/>
       <c r="AH27" t="n">
-        <v>0.5661407329307805</v>
+        <v>0.5661662194924116</v>
       </c>
     </row>
     <row r="28">
@@ -3525,7 +3525,7 @@
       <c r="AF28" t="inlineStr"/>
       <c r="AG28" t="inlineStr"/>
       <c r="AH28" t="n">
-        <v>0.5654406074804039</v>
+        <v>0.5657489081297963</v>
       </c>
     </row>
     <row r="29">
@@ -3635,7 +3635,7 @@
       <c r="AF29" t="inlineStr"/>
       <c r="AG29" t="inlineStr"/>
       <c r="AH29" t="n">
-        <v>0.5649408835628557</v>
+        <v>0.5649465653810375</v>
       </c>
     </row>
     <row r="30">
@@ -3741,7 +3741,7 @@
       <c r="AF30" t="inlineStr"/>
       <c r="AG30" t="inlineStr"/>
       <c r="AH30" t="n">
-        <v>0.5638361949222238</v>
+        <v>0.563861681483855</v>
       </c>
     </row>
     <row r="31">
@@ -3847,7 +3847,7 @@
       <c r="AF31" t="inlineStr"/>
       <c r="AG31" t="inlineStr"/>
       <c r="AH31" t="n">
-        <v>0.5633556051191786</v>
+        <v>0.5633810916808097</v>
       </c>
     </row>
     <row r="32">
@@ -3957,7 +3957,7 @@
       <c r="AF32" t="inlineStr"/>
       <c r="AG32" t="inlineStr"/>
       <c r="AH32" t="n">
-        <v>0.5599323081899694</v>
+        <v>0.5602010822592891</v>
       </c>
     </row>
     <row r="33">
@@ -4173,7 +4173,7 @@
       <c r="AF34" t="inlineStr"/>
       <c r="AG34" t="inlineStr"/>
       <c r="AH34" t="n">
-        <v>0.5522797472762144</v>
+        <v>0.5522354328949435</v>
       </c>
     </row>
     <row r="35">
@@ -4385,7 +4385,7 @@
       <c r="AF36" t="inlineStr"/>
       <c r="AG36" t="inlineStr"/>
       <c r="AH36" t="n">
-        <v>0.549995336928022</v>
+        <v>0.550171262853948</v>
       </c>
     </row>
     <row r="37">
@@ -4497,17 +4497,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>kennalu01</t>
+          <t>smartma01</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>LUKE KENNARD</t>
+          <t>MARCUS SMART</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -4522,102 +4522,102 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H38" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="I38" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J38" t="n">
-        <v>999</v>
+        <v>605</v>
       </c>
       <c r="K38" t="n">
-        <v>429</v>
+        <v>289</v>
       </c>
       <c r="L38" t="n">
-        <v>136</v>
+        <v>86</v>
       </c>
       <c r="M38" t="n">
-        <v>113</v>
+        <v>53</v>
       </c>
       <c r="N38" t="n">
-        <v>20</v>
+        <v>41</v>
       </c>
       <c r="O38" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P38" t="n">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="Q38" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="R38" t="n">
-        <v>0.889</v>
+        <v>0.768</v>
       </c>
       <c r="S38" t="n">
-        <v>0.442</v>
+        <v>0.583</v>
       </c>
       <c r="T38" t="n">
-        <v>0.45</v>
+        <v>0.313</v>
       </c>
       <c r="U38" t="n">
-        <v>0.448</v>
+        <v>0.43</v>
       </c>
       <c r="V38" t="n">
-        <v>887</v>
+        <v>620</v>
       </c>
       <c r="W38" t="n">
-        <v>22.74358974358974</v>
+        <v>31</v>
       </c>
       <c r="X38" t="n">
-        <v>0.8878878878878879</v>
+        <v>1.024793388429752</v>
       </c>
       <c r="Y38" t="n">
-        <v>40.31818181818182</v>
+        <v>31</v>
       </c>
       <c r="Z38" t="n">
-        <v>0.05943446797105334</v>
+        <v>0.04154382203162691</v>
       </c>
       <c r="AA38" t="n">
-        <v>31.96396396396396</v>
+        <v>36.89256198347107</v>
       </c>
       <c r="AB38" t="n">
-        <v>3.154411764705882</v>
+        <v>3.36046511627907</v>
       </c>
       <c r="AC38" t="inlineStr">
         <is>
-          <t>Nivel 3: Above Average</t>
+          <t>Nivel 4: Elite</t>
         </is>
       </c>
       <c r="AD38" t="n">
-        <v>1586</v>
+        <v>2281</v>
       </c>
       <c r="AE38" t="n">
-        <v>-699</v>
+        <v>-1661</v>
       </c>
       <c r="AF38" t="inlineStr"/>
       <c r="AG38" t="inlineStr"/>
       <c r="AH38" t="n">
-        <v>0.5465017240459263</v>
+        <v>0.5465759989597527</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>smartma01</t>
+          <t>kennalu01</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>MARCUS SMART</t>
+          <t>LUKE KENNARD</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -4632,86 +4632,86 @@
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H39" t="n">
+        <v>39</v>
+      </c>
+      <c r="I39" t="n">
+        <v>22</v>
+      </c>
+      <c r="J39" t="n">
+        <v>999</v>
+      </c>
+      <c r="K39" t="n">
+        <v>429</v>
+      </c>
+      <c r="L39" t="n">
+        <v>136</v>
+      </c>
+      <c r="M39" t="n">
+        <v>113</v>
+      </c>
+      <c r="N39" t="n">
         <v>20</v>
       </c>
-      <c r="I39" t="n">
-        <v>20</v>
-      </c>
-      <c r="J39" t="n">
-        <v>605</v>
-      </c>
-      <c r="K39" t="n">
-        <v>289</v>
-      </c>
-      <c r="L39" t="n">
-        <v>86</v>
-      </c>
-      <c r="M39" t="n">
-        <v>53</v>
-      </c>
-      <c r="N39" t="n">
-        <v>41</v>
-      </c>
       <c r="O39" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="P39" t="n">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="Q39" t="n">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="R39" t="n">
-        <v>0.768</v>
+        <v>0.889</v>
       </c>
       <c r="S39" t="n">
-        <v>0.583</v>
+        <v>0.442</v>
       </c>
       <c r="T39" t="n">
-        <v>0.313</v>
+        <v>0.45</v>
       </c>
       <c r="U39" t="n">
-        <v>0.43</v>
+        <v>0.448</v>
       </c>
       <c r="V39" t="n">
-        <v>620</v>
+        <v>887</v>
       </c>
       <c r="W39" t="n">
-        <v>31</v>
+        <v>22.74358974358974</v>
       </c>
       <c r="X39" t="n">
-        <v>1.024793388429752</v>
+        <v>0.8878878878878879</v>
       </c>
       <c r="Y39" t="n">
-        <v>31</v>
+        <v>40.31818181818182</v>
       </c>
       <c r="Z39" t="n">
-        <v>0.04154382203162691</v>
+        <v>0.05943446797105334</v>
       </c>
       <c r="AA39" t="n">
-        <v>36.89256198347107</v>
+        <v>31.96396396396396</v>
       </c>
       <c r="AB39" t="n">
-        <v>3.36046511627907</v>
+        <v>3.154411764705882</v>
       </c>
       <c r="AC39" t="inlineStr">
         <is>
-          <t>Nivel 4: Elite</t>
+          <t>Nivel 3: Above Average</t>
         </is>
       </c>
       <c r="AD39" t="n">
-        <v>2281</v>
+        <v>1586</v>
       </c>
       <c r="AE39" t="n">
-        <v>-1661</v>
+        <v>-699</v>
       </c>
       <c r="AF39" t="inlineStr"/>
       <c r="AG39" t="inlineStr"/>
       <c r="AH39" t="n">
-        <v>0.5462221371711349</v>
+        <v>0.5464088669030691</v>
       </c>
     </row>
     <row r="40">
@@ -4821,7 +4821,7 @@
       <c r="AF40" t="inlineStr"/>
       <c r="AG40" t="inlineStr"/>
       <c r="AH40" t="n">
-        <v>0.5448230702779675</v>
+        <v>0.5448287520961493</v>
       </c>
     </row>
     <row r="41">
@@ -4931,18 +4931,18 @@
       <c r="AF41" t="inlineStr"/>
       <c r="AG41" t="inlineStr"/>
       <c r="AH41" t="n">
-        <v>0.5441968467048691</v>
+        <v>0.544202528523051</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>sharpsh01</t>
+          <t>wallaca01</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SHAEDON SHARPE</t>
+          <t>CASON WALLACE</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -4955,7 +4955,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>POR</t>
+          <t>OKC</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -4965,99 +4965,95 @@
         <v>20</v>
       </c>
       <c r="H42" t="n">
-        <v>32</v>
+        <v>82</v>
       </c>
       <c r="I42" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="J42" t="n">
-        <v>1059</v>
+        <v>1692</v>
       </c>
       <c r="K42" t="n">
-        <v>510</v>
+        <v>561</v>
       </c>
       <c r="L42" t="n">
-        <v>94</v>
+        <v>120</v>
       </c>
       <c r="M42" t="n">
-        <v>160</v>
+        <v>187</v>
       </c>
       <c r="N42" t="n">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="O42" t="n">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="P42" t="n">
-        <v>72</v>
+        <v>45</v>
       </c>
       <c r="Q42" t="n">
-        <v>88</v>
+        <v>129</v>
       </c>
       <c r="R42" t="n">
-        <v>0.824</v>
+        <v>0.784</v>
       </c>
       <c r="S42" t="n">
-        <v>0.457</v>
+        <v>0.572</v>
       </c>
       <c r="T42" t="n">
-        <v>0.333</v>
+        <v>0.419</v>
       </c>
       <c r="U42" t="n">
-        <v>0.406</v>
+        <v>0.491</v>
       </c>
       <c r="V42" t="n">
-        <v>891</v>
+        <v>1470</v>
       </c>
       <c r="W42" t="n">
-        <v>27.84375</v>
+        <v>17.92682926829268</v>
       </c>
       <c r="X42" t="n">
-        <v>0.8413597733711048</v>
+        <v>0.8687943262411347</v>
       </c>
       <c r="Y42" t="n">
-        <v>35.64</v>
+        <v>113.0769230769231</v>
       </c>
       <c r="Z42" t="n">
-        <v>0.05313692748091603</v>
+        <v>0.06936252536214788</v>
       </c>
       <c r="AA42" t="n">
-        <v>30.28895184135977</v>
+        <v>31.27659574468085</v>
       </c>
       <c r="AB42" t="n">
-        <v>5.425531914893617</v>
+        <v>4.675</v>
       </c>
       <c r="AC42" t="inlineStr">
         <is>
           <t>Nivel 3: Above Average</t>
         </is>
       </c>
-      <c r="AD42" t="n">
-        <v>1410</v>
-      </c>
-      <c r="AE42" t="n">
-        <v>-519</v>
-      </c>
+      <c r="AD42" t="inlineStr"/>
+      <c r="AE42" t="inlineStr"/>
       <c r="AF42" t="inlineStr"/>
       <c r="AG42" t="inlineStr"/>
       <c r="AH42" t="n">
-        <v>0.5438712320157384</v>
+        <v>0.5440194051615173</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>jacksis01</t>
+          <t>sharpsh01</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ISAIAH JACKSON</t>
+          <t>SHAEDON SHARPE</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -5065,109 +5061,109 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>IND</t>
+          <t>POR</t>
         </is>
       </c>
       <c r="F43" t="n">
         <v>0</v>
       </c>
       <c r="G43" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H43" t="n">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="I43" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="J43" t="n">
-        <v>771</v>
+        <v>1059</v>
       </c>
       <c r="K43" t="n">
-        <v>383</v>
+        <v>510</v>
       </c>
       <c r="L43" t="n">
-        <v>50</v>
+        <v>94</v>
       </c>
       <c r="M43" t="n">
-        <v>238</v>
+        <v>160</v>
       </c>
       <c r="N43" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="O43" t="n">
-        <v>61</v>
+        <v>12</v>
       </c>
       <c r="P43" t="n">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="Q43" t="n">
-        <v>137</v>
+        <v>88</v>
       </c>
       <c r="R43" t="n">
-        <v>0.716</v>
+        <v>0.824</v>
       </c>
       <c r="S43" t="n">
-        <v>0.677</v>
+        <v>0.457</v>
       </c>
       <c r="T43" t="n">
-        <v>0</v>
+        <v>0.333</v>
       </c>
       <c r="U43" t="n">
-        <v>0.665</v>
+        <v>0.406</v>
       </c>
       <c r="V43" t="n">
-        <v>1075</v>
+        <v>891</v>
       </c>
       <c r="W43" t="n">
-        <v>18.22033898305085</v>
+        <v>27.84375</v>
       </c>
       <c r="X43" t="n">
-        <v>1.394293125810635</v>
+        <v>0.8413597733711048</v>
       </c>
       <c r="Y43" t="n">
-        <v>358.3333333333333</v>
+        <v>35.64</v>
       </c>
       <c r="Z43" t="n">
-        <v>0.05872712373668396</v>
+        <v>0.05313692748091603</v>
       </c>
       <c r="AA43" t="n">
-        <v>50.19455252918288</v>
+        <v>30.28895184135977</v>
       </c>
       <c r="AB43" t="n">
-        <v>7.66</v>
+        <v>5.425531914893617</v>
       </c>
       <c r="AC43" t="inlineStr">
         <is>
-          <t>Nivel 4: Elite</t>
+          <t>Nivel 3: Above Average</t>
         </is>
       </c>
       <c r="AD43" t="n">
-        <v>1234</v>
+        <v>1410</v>
       </c>
       <c r="AE43" t="n">
-        <v>-159</v>
+        <v>-519</v>
       </c>
       <c r="AF43" t="inlineStr"/>
       <c r="AG43" t="inlineStr"/>
       <c r="AH43" t="n">
-        <v>0.5436522664733316</v>
+        <v>0.5438712320157384</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>wallaca01</t>
+          <t>jacksis01</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CASON WALLACE</t>
+          <t>ISAIAH JACKSON</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -5175,89 +5171,93 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>OKC</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="F44" t="n">
         <v>0</v>
       </c>
       <c r="G44" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H44" t="n">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="I44" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="J44" t="n">
-        <v>1692</v>
+        <v>771</v>
       </c>
       <c r="K44" t="n">
-        <v>561</v>
+        <v>383</v>
       </c>
       <c r="L44" t="n">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="M44" t="n">
-        <v>187</v>
+        <v>238</v>
       </c>
       <c r="N44" t="n">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="O44" t="n">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="P44" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="Q44" t="n">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="R44" t="n">
-        <v>0.784</v>
+        <v>0.716</v>
       </c>
       <c r="S44" t="n">
-        <v>0.572</v>
+        <v>0.677</v>
       </c>
       <c r="T44" t="n">
-        <v>0.419</v>
+        <v>0</v>
       </c>
       <c r="U44" t="n">
-        <v>0.491</v>
+        <v>0.665</v>
       </c>
       <c r="V44" t="n">
-        <v>1470</v>
+        <v>1075</v>
       </c>
       <c r="W44" t="n">
-        <v>17.92682926829268</v>
+        <v>18.22033898305085</v>
       </c>
       <c r="X44" t="n">
-        <v>0.8687943262411347</v>
+        <v>1.394293125810635</v>
       </c>
       <c r="Y44" t="n">
-        <v>113.0769230769231</v>
+        <v>358.3333333333333</v>
       </c>
       <c r="Z44" t="n">
-        <v>0.06936252536214788</v>
+        <v>0.05872712373668396</v>
       </c>
       <c r="AA44" t="n">
-        <v>31.27659574468085</v>
+        <v>50.19455252918288</v>
       </c>
       <c r="AB44" t="n">
-        <v>4.675</v>
+        <v>7.66</v>
       </c>
       <c r="AC44" t="inlineStr">
         <is>
-          <t>Nivel 3: Above Average</t>
-        </is>
-      </c>
-      <c r="AD44" t="inlineStr"/>
-      <c r="AE44" t="inlineStr"/>
+          <t>Nivel 4: Elite</t>
+        </is>
+      </c>
+      <c r="AD44" t="n">
+        <v>1234</v>
+      </c>
+      <c r="AE44" t="n">
+        <v>-159</v>
+      </c>
       <c r="AF44" t="inlineStr"/>
       <c r="AG44" t="inlineStr"/>
       <c r="AH44" t="n">
-        <v>0.5435637195427881</v>
+        <v>0.5436522664733316</v>
       </c>
     </row>
     <row r="45">
@@ -5689,7 +5689,7 @@
       <c r="AF48" t="inlineStr"/>
       <c r="AG48" t="inlineStr"/>
       <c r="AH48" t="n">
-        <v>0.5396222334544123</v>
+        <v>0.5396477200160434</v>
       </c>
     </row>
     <row r="49">
@@ -5799,18 +5799,18 @@
       <c r="AF49" t="inlineStr"/>
       <c r="AG49" t="inlineStr"/>
       <c r="AH49" t="n">
-        <v>0.5392128836984191</v>
+        <v>0.5393069745530279</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>jacksan01</t>
+          <t>jonesco02</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ANDRE JACKSON JR.</t>
+          <t>COLBY JONES</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -5823,81 +5823,81 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>MIL</t>
+          <t>SAC</t>
         </is>
       </c>
       <c r="F50" t="n">
         <v>0</v>
       </c>
       <c r="G50" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H50" t="n">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="I50" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>572</v>
+        <v>192</v>
       </c>
       <c r="K50" t="n">
-        <v>125</v>
+        <v>64</v>
       </c>
       <c r="L50" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="M50" t="n">
-        <v>113</v>
+        <v>40</v>
       </c>
       <c r="N50" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="O50" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="P50" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="Q50" t="n">
-        <v>92</v>
+        <v>29</v>
       </c>
       <c r="R50" t="n">
-        <v>0.727</v>
+        <v>0.545</v>
       </c>
       <c r="S50" t="n">
-        <v>0.611</v>
+        <v>0.531</v>
       </c>
       <c r="T50" t="n">
-        <v>0.37</v>
+        <v>0.091</v>
       </c>
       <c r="U50" t="n">
-        <v>0.5</v>
+        <v>0.394</v>
       </c>
       <c r="V50" t="n">
-        <v>396</v>
+        <v>172</v>
       </c>
       <c r="W50" t="n">
-        <v>6.947368421052632</v>
+        <v>5.733333333333333</v>
       </c>
       <c r="X50" t="n">
-        <v>0.6923076923076923</v>
+        <v>0.8958333333333334</v>
       </c>
       <c r="Y50" t="n">
-        <v>49.5</v>
+        <v>0</v>
       </c>
       <c r="Z50" t="n">
-        <v>0.02015985338288449</v>
+        <v>0.008238731618527567</v>
       </c>
       <c r="AA50" t="n">
-        <v>24.92307692307692</v>
+        <v>32.25</v>
       </c>
       <c r="AB50" t="n">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="AC50" t="inlineStr">
         <is>
-          <t>Nivel 2: Average</t>
+          <t>Nivel 3: Above Average</t>
         </is>
       </c>
       <c r="AD50" t="inlineStr"/>
@@ -5905,18 +5905,18 @@
       <c r="AF50" t="inlineStr"/>
       <c r="AG50" t="inlineStr"/>
       <c r="AH50" t="n">
-        <v>0.5363264118556926</v>
+        <v>0.5363726156744538</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>jonesco02</t>
+          <t>jacksan01</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>COLBY JONES</t>
+          <t>ANDRE JACKSON JR.</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -5929,81 +5929,81 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>SAC</t>
+          <t>MIL</t>
         </is>
       </c>
       <c r="F51" t="n">
         <v>0</v>
       </c>
       <c r="G51" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H51" t="n">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="I51" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J51" t="n">
-        <v>192</v>
+        <v>572</v>
       </c>
       <c r="K51" t="n">
-        <v>64</v>
+        <v>125</v>
       </c>
       <c r="L51" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="M51" t="n">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="N51" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="O51" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P51" t="n">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="Q51" t="n">
-        <v>29</v>
+        <v>92</v>
       </c>
       <c r="R51" t="n">
-        <v>0.545</v>
+        <v>0.727</v>
       </c>
       <c r="S51" t="n">
-        <v>0.531</v>
+        <v>0.611</v>
       </c>
       <c r="T51" t="n">
-        <v>0.091</v>
+        <v>0.37</v>
       </c>
       <c r="U51" t="n">
-        <v>0.394</v>
+        <v>0.5</v>
       </c>
       <c r="V51" t="n">
-        <v>172</v>
+        <v>396</v>
       </c>
       <c r="W51" t="n">
-        <v>5.733333333333333</v>
+        <v>6.947368421052632</v>
       </c>
       <c r="X51" t="n">
-        <v>0.8958333333333334</v>
+        <v>0.6923076923076923</v>
       </c>
       <c r="Y51" t="n">
-        <v>0</v>
+        <v>49.5</v>
       </c>
       <c r="Z51" t="n">
-        <v>0.008238731618527567</v>
+        <v>0.02015985338288449</v>
       </c>
       <c r="AA51" t="n">
-        <v>32.25</v>
+        <v>24.92307692307692</v>
       </c>
       <c r="AB51" t="n">
-        <v>3.2</v>
+        <v>2.5</v>
       </c>
       <c r="AC51" t="inlineStr">
         <is>
-          <t>Nivel 3: Above Average</t>
+          <t>Nivel 2: Average</t>
         </is>
       </c>
       <c r="AD51" t="inlineStr"/>
@@ -6011,7 +6011,7 @@
       <c r="AF51" t="inlineStr"/>
       <c r="AG51" t="inlineStr"/>
       <c r="AH51" t="n">
-        <v>0.5358854523747906</v>
+        <v>0.5363264118556926</v>
       </c>
     </row>
   </sheetData>

</xml_diff>